<commit_message>
Update IESO report from GitHub Actions
</commit_message>
<xml_diff>
--- a/output/latest.xlsx
+++ b/output/latest.xlsx
@@ -493,7 +493,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>CreatedAt: 2026-09-21T23:11:16</t>
+          <t>CreatedAt: 2026-09-22T04:10:26</t>
         </is>
       </c>
       <c r="B1" s="3" t="n"/>
@@ -653,70 +653,70 @@
         <v>20.71</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>54.44</v>
+        <v>20.62</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>20.64</v>
+        <v>56.06</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>33.05</v>
+        <v>20.46</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>45.5</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>44.9</v>
+        <v>80.13</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>39.63</v>
+        <v>51.22</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>35.24</v>
+        <v>34.58</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>31.28</v>
+        <v>31.53</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>31.28</v>
+        <v>31.61</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>31.56</v>
+        <v>34.04</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>32.27</v>
+        <v>34.04</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>32.24</v>
+        <v>33.97</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>39.67</v>
+        <v>33.9</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>46.52</v>
+        <v>39.71</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>54.05</v>
+        <v>47.53</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>53.84</v>
+        <v>49.49</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>51.45</v>
+        <v>47.52</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>46.56</v>
+        <v>47.61</v>
       </c>
       <c r="V4" s="3" t="n">
-        <v>35.83</v>
+        <v>47.38</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>33.76</v>
+        <v>45.11</v>
       </c>
       <c r="X4" s="3" t="n">
-        <v>31.22</v>
+        <v>35.66</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>36.35</v>
+        <v>43.19</v>
       </c>
       <c r="Z4" s="3" t="n">
         <v>38.96</v>
@@ -824,70 +824,70 @@
         <v>0.12</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.14</v>
+        <v>0.09</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="K6" s="3" t="n">
         <v>-0.32</v>
       </c>
-      <c r="H6" s="3" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>-0.31</v>
-      </c>
       <c r="L6" s="3" t="n">
-        <v>-0.31</v>
+        <v>-0.28</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>-0.25</v>
+        <v>-0.2</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.1</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>-0.23</v>
+        <v>-0.14</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>-0.32</v>
+        <v>-0.2</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.2</v>
       </c>
       <c r="R6" s="3" t="n">
-        <v>-0.92</v>
+        <v>-0.52</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>-1.08</v>
+        <v>-0.95</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>-1.07</v>
+        <v>-1.19</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>-0.47</v>
+        <v>-1.04</v>
       </c>
       <c r="W6" s="3" t="n">
-        <v>-0.14</v>
+        <v>-0.68</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.39</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>-0.33</v>
+        <v>-0.43</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>-0.55</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="7">
@@ -905,19 +905,19 @@
         <v>0</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>33.82</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0</v>
+        <v>40.86</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0</v>
+        <v>36.47</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>0</v>
+        <v>43.32</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>0</v>
@@ -1073,73 +1073,73 @@
         <v>21.39</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>21.55</v>
+        <v>21.57</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>21.44</v>
+        <v>16.03</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>34.15</v>
+        <v>21.61</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>46.42</v>
+        <v>32.59</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>45.76</v>
+        <v>37.64</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>40.47</v>
+        <v>52.53</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>35.8</v>
+        <v>35.46</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>32.14</v>
+        <v>32.3</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>32.3</v>
+        <v>32.98</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>32.53</v>
+        <v>35.78</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>33.13</v>
+        <v>35.23</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>33.23</v>
+        <v>35.38</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>40.68</v>
+        <v>35.23</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>48.19</v>
+        <v>41.61</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>55.75</v>
+        <v>49.54</v>
       </c>
       <c r="S9" s="3" t="n">
-        <v>55.43</v>
+        <v>51.16</v>
       </c>
       <c r="T9" s="3" t="n">
-        <v>53.38</v>
+        <v>49.16</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>48.6</v>
+        <v>49.59</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>37.38</v>
+        <v>49.26</v>
       </c>
       <c r="W9" s="3" t="n">
-        <v>35.24</v>
+        <v>47.31</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>32.21</v>
+        <v>36.71</v>
       </c>
       <c r="Y9" s="3" t="n">
-        <v>37.08</v>
+        <v>44.33</v>
       </c>
       <c r="Z9" s="3" t="n">
-        <v>39.58</v>
+        <v>39.62</v>
       </c>
     </row>
     <row r="10">
@@ -1241,70 +1241,70 @@
         <v>0.73</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.2</v>
+        <v>1.34</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.6</v>
+        <v>0.88</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>0.32</v>
+        <v>0.75</v>
       </c>
       <c r="I11" s="3" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="K11" s="3" t="n">
         <v>0.45</v>
       </c>
-      <c r="J11" s="3" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="K11" s="3" t="n">
-        <v>0.55</v>
-      </c>
       <c r="L11" s="3" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="S11" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="T11" s="3" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="U11" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="X11" s="3" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="Y11" s="3" t="n">
         <v>0.71</v>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="O11" s="3" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="Q11" s="3" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="R11" s="3" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="S11" s="3" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="T11" s="3" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="U11" s="3" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="V11" s="3" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="W11" s="3" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="X11" s="3" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="Y11" s="3" t="n">
-        <v>0.41</v>
       </c>
       <c r="Z11" s="3" t="n">
         <v>0.08</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>0</v>
@@ -1493,73 +1493,73 @@
         <v>21.39</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>21.55</v>
+        <v>21.57</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>21.44</v>
+        <v>23.61</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>34.15</v>
+        <v>26.52</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>46.42</v>
+        <v>32.59</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>45.76</v>
+        <v>37.64</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>40.51</v>
+        <v>52.58</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>35.8</v>
+        <v>35.5</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>32.14</v>
+        <v>36.53</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>36.55</v>
+        <v>37.37</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>36.9</v>
+        <v>35.78</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>37.33</v>
+        <v>39.91</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>37.45</v>
+        <v>40.1</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>46.25</v>
+        <v>40.03</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>48.24</v>
+        <v>47.31</v>
       </c>
       <c r="R14" s="3" t="n">
-        <v>63.79</v>
+        <v>56.63</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>63.48</v>
+        <v>58.48</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>61</v>
+        <v>55.93</v>
       </c>
       <c r="U14" s="3" t="n">
-        <v>55.44</v>
+        <v>56.53</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>42.31</v>
+        <v>56.12</v>
       </c>
       <c r="W14" s="3" t="n">
-        <v>39.96</v>
+        <v>54.44</v>
       </c>
       <c r="X14" s="3" t="n">
-        <v>36.35</v>
+        <v>41.6</v>
       </c>
       <c r="Y14" s="3" t="n">
-        <v>37.08</v>
+        <v>50.46</v>
       </c>
       <c r="Z14" s="3" t="n">
-        <v>39.58</v>
+        <v>39.62</v>
       </c>
     </row>
     <row r="15">
@@ -1580,10 +1580,10 @@
         <v>0</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>4.89</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>0</v>
@@ -1598,49 +1598,49 @@
         <v>0</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>4.22</v>
+        <v>4.38</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>4.37</v>
+        <v>0</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>4.2</v>
+        <v>4.64</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>4.22</v>
+        <v>4.68</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>5.58</v>
+        <v>4.8</v>
       </c>
       <c r="Q15" s="3" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>7.99</v>
+        <v>7.04</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>8.06</v>
+        <v>7.33</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>7.57</v>
+        <v>6.78</v>
       </c>
       <c r="U15" s="3" t="n">
-        <v>6.79</v>
+        <v>6.93</v>
       </c>
       <c r="V15" s="3" t="n">
-        <v>4.93</v>
+        <v>6.86</v>
       </c>
       <c r="W15" s="3" t="n">
-        <v>4.73</v>
+        <v>7.13</v>
       </c>
       <c r="X15" s="3" t="n">
-        <v>4.14</v>
+        <v>4.89</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>0</v>
+        <v>6.13</v>
       </c>
       <c r="Z15" s="3" t="n">
         <v>0</v>
@@ -1661,70 +1661,70 @@
         <v>0.73</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1.06</v>
+        <v>1.08</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1.2</v>
+        <v>1.36</v>
       </c>
       <c r="G16" s="3" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="J16" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="H16" s="3" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>0.14</v>
-      </c>
       <c r="K16" s="3" t="n">
-        <v>0.55</v>
+        <v>0.48</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>0.74</v>
+        <v>1.09</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>0.72</v>
+        <v>1.54</v>
       </c>
       <c r="N16" s="3" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="S16" s="3" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="T16" s="3" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="U16" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="V16" s="3" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="W16" s="3" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="X16" s="3" t="n">
         <v>0.66</v>
       </c>
-      <c r="O16" s="3" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="P16" s="3" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="Q16" s="3" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="R16" s="3" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="S16" s="3" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="T16" s="3" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="U16" s="3" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="V16" s="3" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="W16" s="3" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="X16" s="3" t="n">
-        <v>0.84</v>
-      </c>
       <c r="Y16" s="3" t="n">
-        <v>0.41</v>
+        <v>0.71</v>
       </c>
       <c r="Z16" s="3" t="n">
         <v>0.08</v>
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J18" s="3" t="n">
         <v>0</v>
@@ -1913,73 +1913,73 @@
         <v>63.24</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>60.22</v>
+        <v>60.24</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>20.68</v>
+        <v>57.03</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>33.09</v>
+        <v>59.06</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>45.41</v>
+        <v>66.09</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>44.81</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>39.63</v>
+        <v>87.83</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>35.27</v>
+        <v>34.62</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>31.34</v>
+        <v>31.56</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>31.37</v>
+        <v>31.67</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>31.62</v>
+        <v>34.1</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>32.33</v>
+        <v>34.07</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>32.3</v>
+        <v>34.04</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>39.67</v>
+        <v>33.94</v>
       </c>
       <c r="Q19" s="3" t="n">
-        <v>46.52</v>
+        <v>39.75</v>
       </c>
       <c r="R19" s="3" t="n">
-        <v>53.99</v>
+        <v>47.48</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>53.74</v>
+        <v>49.44</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>51.4</v>
+        <v>47.47</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>46.51</v>
+        <v>47.56</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>35.79</v>
+        <v>47.29</v>
       </c>
       <c r="W19" s="3" t="n">
-        <v>33.8</v>
+        <v>45.07</v>
       </c>
       <c r="X19" s="3" t="n">
-        <v>31.28</v>
+        <v>35.66</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>36.35</v>
+        <v>43.14</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>39.07</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20">
@@ -2081,73 +2081,73 @@
         <v>0.06</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.19</v>
+        <v>0.12</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.03</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.11</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>-0.4</v>
+        <v>-0.18</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>-0.39</v>
+        <v>-0.28</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>-0.25</v>
+        <v>-0.28</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>-0.22</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>-0.13</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="O21" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="Q21" s="3" t="n">
         <v>-0.16</v>
       </c>
-      <c r="P21" s="3" t="n">
-        <v>-0.32</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>-0.6</v>
-      </c>
       <c r="R21" s="3" t="n">
-        <v>-0.97</v>
+        <v>-0.57</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>-0.91</v>
+        <v>-0.74</v>
       </c>
       <c r="T21" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U21" s="3" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="V21" s="3" t="n">
         <v>-1.13</v>
       </c>
-      <c r="U21" s="3" t="n">
-        <v>-1.12</v>
-      </c>
-      <c r="V21" s="3" t="n">
-        <v>-0.5</v>
-      </c>
       <c r="W21" s="3" t="n">
-        <v>-0.1</v>
+        <v>-0.72</v>
       </c>
       <c r="X21" s="3" t="n">
-        <v>-0.09</v>
+        <v>-0.39</v>
       </c>
       <c r="Y21" s="3" t="n">
-        <v>-0.33</v>
+        <v>-0.47</v>
       </c>
       <c r="Z21" s="3" t="n">
-        <v>-0.43</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="22">
@@ -2165,22 +2165,22 @@
         <v>42.51</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>39.54</v>
+        <v>39.58</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>41.8</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0</v>
+        <v>38.54</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>0</v>
+        <v>34.42</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>0</v>
+        <v>61.57</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>0</v>
+        <v>36.65</v>
       </c>
       <c r="J22" s="3" t="n">
         <v>0</v>
@@ -2264,7 +2264,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J23" s="3" t="n">
         <v>0</v>
@@ -2333,73 +2333,73 @@
         <v>20.73</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>54.5</v>
+        <v>20.66</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>20.68</v>
+        <v>56.09</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>33.09</v>
+        <v>20.52</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>45.41</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>44.81</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>39.63</v>
+        <v>51.18</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>35.27</v>
+        <v>34.62</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>31.34</v>
+        <v>31.56</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>31.37</v>
+        <v>31.67</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>31.62</v>
+        <v>34.1</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>32.33</v>
+        <v>34.07</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>32.3</v>
+        <v>34.04</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>39.67</v>
+        <v>33.94</v>
       </c>
       <c r="Q24" s="3" t="n">
-        <v>46.52</v>
+        <v>39.75</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>53.99</v>
+        <v>47.48</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>53.74</v>
+        <v>49.44</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>51.4</v>
+        <v>47.47</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>46.51</v>
+        <v>47.56</v>
       </c>
       <c r="V24" s="3" t="n">
-        <v>35.79</v>
+        <v>47.29</v>
       </c>
       <c r="W24" s="3" t="n">
-        <v>33.8</v>
+        <v>45.07</v>
       </c>
       <c r="X24" s="3" t="n">
-        <v>31.28</v>
+        <v>35.66</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>36.35</v>
+        <v>43.14</v>
       </c>
       <c r="Z24" s="3" t="n">
-        <v>39.07</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25">
@@ -2501,73 +2501,73 @@
         <v>0.06</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.19</v>
+        <v>0.12</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-0.41</v>
+        <v>-0.03</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>-0.63</v>
+        <v>-0.11</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>-0.4</v>
+        <v>-0.18</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>-0.39</v>
+        <v>-0.28</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>-0.25</v>
+        <v>-0.28</v>
       </c>
       <c r="L26" s="3" t="n">
         <v>-0.22</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>-0.13</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="O26" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="Q26" s="3" t="n">
         <v>-0.16</v>
       </c>
-      <c r="P26" s="3" t="n">
-        <v>-0.32</v>
-      </c>
-      <c r="Q26" s="3" t="n">
-        <v>-0.6</v>
-      </c>
       <c r="R26" s="3" t="n">
-        <v>-0.97</v>
+        <v>-0.57</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>-0.91</v>
+        <v>-0.74</v>
       </c>
       <c r="T26" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="U26" s="3" t="n">
+        <v>-1.24</v>
+      </c>
+      <c r="V26" s="3" t="n">
         <v>-1.13</v>
       </c>
-      <c r="U26" s="3" t="n">
-        <v>-1.12</v>
-      </c>
-      <c r="V26" s="3" t="n">
-        <v>-0.5</v>
-      </c>
       <c r="W26" s="3" t="n">
-        <v>-0.1</v>
+        <v>-0.72</v>
       </c>
       <c r="X26" s="3" t="n">
-        <v>-0.09</v>
+        <v>-0.39</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>-0.33</v>
+        <v>-0.47</v>
       </c>
       <c r="Z26" s="3" t="n">
-        <v>-0.43</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="27">
@@ -2585,19 +2585,19 @@
         <v>0</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>33.82</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0</v>
+        <v>40.86</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>0</v>
+        <v>36.47</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>0</v>
+        <v>43.32</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>0</v>
@@ -2684,7 +2684,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J28" s="3" t="n">
         <v>0</v>
@@ -2756,70 +2756,70 @@
         <v>60.2</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>20.68</v>
+        <v>57</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>33.02</v>
+        <v>59</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>45.23</v>
+        <v>66</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>44.59</v>
+        <v>98.2</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>39.51</v>
+        <v>87.61</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>35.2</v>
+        <v>34.55</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>31.31</v>
+        <v>31.5</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>31.31</v>
+        <v>31.58</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>31.59</v>
+        <v>34</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>32.27</v>
+        <v>33.97</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>32.27</v>
+        <v>33.97</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>39.55</v>
+        <v>33.83</v>
       </c>
       <c r="Q29" s="3" t="n">
-        <v>46.29</v>
+        <v>39.59</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>53.73</v>
+        <v>47.29</v>
       </c>
       <c r="S29" s="3" t="n">
-        <v>53.53</v>
+        <v>49.2</v>
       </c>
       <c r="T29" s="3" t="n">
-        <v>51.15</v>
+        <v>47.24</v>
       </c>
       <c r="U29" s="3" t="n">
-        <v>46.29</v>
+        <v>47.42</v>
       </c>
       <c r="V29" s="3" t="n">
-        <v>35.65</v>
+        <v>46.97</v>
       </c>
       <c r="W29" s="3" t="n">
-        <v>33.7</v>
+        <v>44.81</v>
       </c>
       <c r="X29" s="3" t="n">
-        <v>31.22</v>
+        <v>35.55</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>36.2</v>
+        <v>42.93</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>39.15</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="30">
@@ -2921,73 +2921,73 @@
         <v>0.02</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.19</v>
+        <v>0.09</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-0.59</v>
+        <v>-0.13</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>-0.85</v>
+        <v>-0.26</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>-0.51</v>
+        <v>-0.39</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>-0.46</v>
+        <v>-0.35</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.35</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.32</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>-0.22</v>
+        <v>-0.24</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.17</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.27</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>-0.83</v>
+        <v>-0.32</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>-1.24</v>
+        <v>-0.76</v>
       </c>
       <c r="S31" s="3" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="T31" s="3" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="U31" s="3" t="n">
         <v>-1.38</v>
       </c>
-      <c r="U31" s="3" t="n">
-        <v>-1.34</v>
-      </c>
       <c r="V31" s="3" t="n">
-        <v>-0.64</v>
+        <v>-1.46</v>
       </c>
       <c r="W31" s="3" t="n">
-        <v>-0.2</v>
+        <v>-0.99</v>
       </c>
       <c r="X31" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.5</v>
       </c>
       <c r="Y31" s="3" t="n">
-        <v>-0.47</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="Z31" s="3" t="n">
-        <v>-0.35</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="32">
@@ -3005,22 +3005,22 @@
         <v>42.51</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>39.54</v>
+        <v>39.58</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0</v>
+        <v>41.8</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>0</v>
+        <v>38.54</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>0</v>
+        <v>34.42</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>0</v>
+        <v>61.57</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>0</v>
+        <v>36.65</v>
       </c>
       <c r="J32" s="3" t="n">
         <v>0</v>
@@ -3104,7 +3104,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>0</v>
@@ -3173,73 +3173,73 @@
         <v>21.85</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>22.11</v>
+        <v>22.13</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>21.92</v>
+        <v>24.08</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>34.91</v>
+        <v>27.17</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>47.28</v>
+        <v>33.24</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>46.65</v>
+        <v>38.38</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>41.26</v>
+        <v>53.49</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>36.24</v>
+        <v>36.05</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>32.7</v>
+        <v>37.17</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>37.16</v>
+        <v>38.24</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>37.48</v>
+        <v>36.86</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>37.85</v>
+        <v>40.69</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>38.11</v>
+        <v>41.04</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>46.97</v>
+        <v>40.96</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>49.35</v>
+        <v>48.52</v>
       </c>
       <c r="R34" s="3" t="n">
-        <v>65.06999999999999</v>
+        <v>58.05</v>
       </c>
       <c r="S34" s="3" t="n">
-        <v>64.69</v>
+        <v>59.71</v>
       </c>
       <c r="T34" s="3" t="n">
-        <v>62.4</v>
+        <v>57.06</v>
       </c>
       <c r="U34" s="3" t="n">
-        <v>56.82</v>
+        <v>57.93</v>
       </c>
       <c r="V34" s="3" t="n">
-        <v>43.34</v>
+        <v>57.52</v>
       </c>
       <c r="W34" s="3" t="n">
-        <v>40.87</v>
+        <v>55.95</v>
       </c>
       <c r="X34" s="3" t="n">
-        <v>36.99</v>
+        <v>42.48</v>
       </c>
       <c r="Y34" s="3" t="n">
-        <v>37.73</v>
+        <v>51.42</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>40.19</v>
+        <v>40.39</v>
       </c>
     </row>
     <row r="35">
@@ -3260,10 +3260,10 @@
         <v>0</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0</v>
+        <v>7.58</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>0</v>
+        <v>4.89</v>
       </c>
       <c r="G35" s="3" t="n">
         <v>0</v>
@@ -3278,49 +3278,49 @@
         <v>0</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0</v>
+        <v>4.2</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>4.22</v>
+        <v>4.38</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>4.37</v>
+        <v>0</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>4.2</v>
+        <v>4.64</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>4.22</v>
+        <v>4.68</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>5.58</v>
+        <v>4.8</v>
       </c>
       <c r="Q35" s="3" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>7.99</v>
+        <v>7.04</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>8.06</v>
+        <v>7.33</v>
       </c>
       <c r="T35" s="3" t="n">
-        <v>7.57</v>
+        <v>6.78</v>
       </c>
       <c r="U35" s="3" t="n">
-        <v>6.79</v>
+        <v>6.93</v>
       </c>
       <c r="V35" s="3" t="n">
-        <v>4.93</v>
+        <v>6.86</v>
       </c>
       <c r="W35" s="3" t="n">
-        <v>4.73</v>
+        <v>7.13</v>
       </c>
       <c r="X35" s="3" t="n">
-        <v>4.14</v>
+        <v>4.89</v>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>0</v>
+        <v>6.13</v>
       </c>
       <c r="Z35" s="3" t="n">
         <v>0</v>
@@ -3341,73 +3341,73 @@
         <v>1.18</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1.61</v>
+        <v>1.64</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>1.42</v>
+        <v>1.4</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1.47</v>
+        <v>1.53</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1.21</v>
+        <v>1.5</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>1.24</v>
+        <v>2.13</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>0.58</v>
+        <v>1.15</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>1.35</v>
+        <v>1.96</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>1.29</v>
+        <v>2.62</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>1.18</v>
+        <v>1.91</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>1.42</v>
+        <v>2.25</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>1.41</v>
+        <v>2.06</v>
       </c>
       <c r="Q36" s="3" t="n">
-        <v>2.22</v>
+        <v>2.91</v>
       </c>
       <c r="R36" s="3" t="n">
-        <v>2.11</v>
+        <v>2.96</v>
       </c>
       <c r="S36" s="3" t="n">
-        <v>1.98</v>
+        <v>2.2</v>
       </c>
       <c r="T36" s="3" t="n">
-        <v>2.3</v>
+        <v>1.81</v>
       </c>
       <c r="U36" s="3" t="n">
-        <v>2.4</v>
+        <v>2.19</v>
       </c>
       <c r="V36" s="3" t="n">
-        <v>2.11</v>
+        <v>2.23</v>
       </c>
       <c r="W36" s="3" t="n">
-        <v>2.24</v>
+        <v>3.03</v>
       </c>
       <c r="X36" s="3" t="n">
-        <v>1.48</v>
+        <v>1.54</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>1.06</v>
+        <v>1.68</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>0.68</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="37">
@@ -3524,7 +3524,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J38" s="3" t="n">
         <v>0</v>
@@ -3593,70 +3593,70 @@
         <v>20.71</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>54.44</v>
+        <v>20.62</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>20.64</v>
+        <v>56.06</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>33.05</v>
+        <v>20.46</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>45.5</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>44.9</v>
+        <v>80.13</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>39.63</v>
+        <v>51.22</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>35.24</v>
+        <v>34.58</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>31.28</v>
+        <v>31.53</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>31.28</v>
+        <v>31.61</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>31.56</v>
+        <v>34.04</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>32.27</v>
+        <v>34.04</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>32.24</v>
+        <v>33.97</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>39.67</v>
+        <v>33.9</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>46.52</v>
+        <v>39.71</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>54.05</v>
+        <v>47.53</v>
       </c>
       <c r="S39" s="3" t="n">
-        <v>53.84</v>
+        <v>49.49</v>
       </c>
       <c r="T39" s="3" t="n">
-        <v>51.45</v>
+        <v>47.52</v>
       </c>
       <c r="U39" s="3" t="n">
-        <v>46.56</v>
+        <v>47.61</v>
       </c>
       <c r="V39" s="3" t="n">
-        <v>35.83</v>
+        <v>47.38</v>
       </c>
       <c r="W39" s="3" t="n">
-        <v>33.76</v>
+        <v>45.11</v>
       </c>
       <c r="X39" s="3" t="n">
-        <v>31.22</v>
+        <v>35.66</v>
       </c>
       <c r="Y39" s="3" t="n">
-        <v>36.35</v>
+        <v>43.19</v>
       </c>
       <c r="Z39" s="3" t="n">
         <v>38.96</v>
@@ -3764,70 +3764,70 @@
         <v>0.12</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0.14</v>
+        <v>0.09</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="G41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="K41" s="3" t="n">
         <v>-0.32</v>
       </c>
-      <c r="H41" s="3" t="n">
-        <v>-0.54</v>
-      </c>
-      <c r="I41" s="3" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="J41" s="3" t="n">
-        <v>-0.42</v>
-      </c>
-      <c r="K41" s="3" t="n">
-        <v>-0.31</v>
-      </c>
       <c r="L41" s="3" t="n">
-        <v>-0.31</v>
+        <v>-0.28</v>
       </c>
       <c r="M41" s="3" t="n">
-        <v>-0.25</v>
+        <v>-0.2</v>
       </c>
       <c r="N41" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.1</v>
       </c>
       <c r="O41" s="3" t="n">
-        <v>-0.23</v>
+        <v>-0.14</v>
       </c>
       <c r="P41" s="3" t="n">
-        <v>-0.32</v>
+        <v>-0.2</v>
       </c>
       <c r="Q41" s="3" t="n">
-        <v>-0.6</v>
+        <v>-0.2</v>
       </c>
       <c r="R41" s="3" t="n">
-        <v>-0.92</v>
+        <v>-0.52</v>
       </c>
       <c r="S41" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="T41" s="3" t="n">
-        <v>-1.08</v>
+        <v>-0.95</v>
       </c>
       <c r="U41" s="3" t="n">
-        <v>-1.07</v>
+        <v>-1.19</v>
       </c>
       <c r="V41" s="3" t="n">
-        <v>-0.47</v>
+        <v>-1.04</v>
       </c>
       <c r="W41" s="3" t="n">
-        <v>-0.14</v>
+        <v>-0.68</v>
       </c>
       <c r="X41" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.39</v>
       </c>
       <c r="Y41" s="3" t="n">
-        <v>-0.33</v>
+        <v>-0.43</v>
       </c>
       <c r="Z41" s="3" t="n">
-        <v>-0.55</v>
+        <v>-0.58</v>
       </c>
     </row>
     <row r="42">
@@ -3845,19 +3845,19 @@
         <v>0</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>33.82</v>
+        <v>0</v>
       </c>
       <c r="E42" s="3" t="n">
-        <v>0</v>
+        <v>40.86</v>
       </c>
       <c r="F42" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G42" s="3" t="n">
-        <v>0</v>
+        <v>36.47</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>0</v>
+        <v>43.32</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>0</v>
@@ -3944,7 +3944,7 @@
         <v>0</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J43" s="3" t="n">
         <v>0</v>
@@ -4013,73 +4013,73 @@
         <v>20.75</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>20.59</v>
+        <v>20.68</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>20.59</v>
+        <v>15.21</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>33.09</v>
+        <v>20.46</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>45.86</v>
+        <v>32</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>45.53</v>
+        <v>37.18</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>39.86</v>
+        <v>51.62</v>
       </c>
       <c r="J44" s="3" t="n">
-        <v>35.31</v>
+        <v>34.72</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>31.34</v>
+        <v>31.69</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>31.25</v>
+        <v>31.61</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>31.47</v>
+        <v>34.04</v>
       </c>
       <c r="N44" s="3" t="n">
-        <v>32.21</v>
+        <v>34.07</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>32.24</v>
+        <v>34.1</v>
       </c>
       <c r="P44" s="3" t="n">
-        <v>39.79</v>
+        <v>34.1</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>46.89</v>
+        <v>40.03</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>55.02</v>
+        <v>48.24</v>
       </c>
       <c r="S44" s="3" t="n">
-        <v>54.81</v>
+        <v>50.39</v>
       </c>
       <c r="T44" s="3" t="n">
-        <v>52.69</v>
+        <v>48.66</v>
       </c>
       <c r="U44" s="3" t="n">
-        <v>47.68</v>
+        <v>48.9</v>
       </c>
       <c r="V44" s="3" t="n">
-        <v>36.44</v>
+        <v>48.57</v>
       </c>
       <c r="W44" s="3" t="n">
-        <v>34.1</v>
+        <v>45.98</v>
       </c>
       <c r="X44" s="3" t="n">
-        <v>31.31</v>
+        <v>35.94</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>36.6</v>
+        <v>43.66</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>39.35</v>
+        <v>39.47</v>
       </c>
     </row>
     <row r="45">
@@ -4181,73 +4181,73 @@
         <v>0.08</v>
       </c>
       <c r="D46" s="3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="L46" s="3" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="M46" s="3" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="3" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="S46" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T46" s="3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="U46" s="3" t="n">
         <v>0.1</v>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="G46" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H46" s="3" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="I46" s="3" t="n">
-        <v>-0.16</v>
-      </c>
-      <c r="J46" s="3" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="K46" s="3" t="n">
-        <v>-0.25</v>
-      </c>
-      <c r="L46" s="3" t="n">
-        <v>-0.34</v>
-      </c>
-      <c r="M46" s="3" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="N46" s="3" t="n">
-        <v>-0.26</v>
-      </c>
-      <c r="O46" s="3" t="n">
-        <v>-0.23</v>
-      </c>
-      <c r="P46" s="3" t="n">
-        <v>-0.2</v>
-      </c>
-      <c r="Q46" s="3" t="n">
-        <v>-0.23</v>
-      </c>
-      <c r="R46" s="3" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="S46" s="3" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="T46" s="3" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U46" s="3" t="n">
-        <v>0.05</v>
       </c>
       <c r="V46" s="3" t="n">
         <v>0.15</v>
       </c>
       <c r="W46" s="3" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="X46" s="3" t="n">
-        <v>-0.06</v>
+        <v>-0.11</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.04</v>
       </c>
       <c r="Z46" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="47">
@@ -4364,7 +4364,7 @@
         <v>0</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J48" s="3" t="n">
         <v>0</v>
@@ -4433,73 +4433,73 @@
         <v>21.31</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>21.06</v>
+        <v>20.93</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>21.04</v>
+        <v>15.51</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>34.08</v>
+        <v>20.81</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>47.77</v>
+        <v>32.89</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>47.63</v>
+        <v>37.45</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>41.35</v>
+        <v>51.8</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>36.46</v>
+        <v>35.04</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>32.23</v>
+        <v>31.91</v>
       </c>
       <c r="L49" s="3" t="n">
-        <v>32.1</v>
+        <v>31.9</v>
       </c>
       <c r="M49" s="3" t="n">
-        <v>32.73</v>
+        <v>34.83</v>
       </c>
       <c r="N49" s="3" t="n">
-        <v>33.4</v>
+        <v>34.66</v>
       </c>
       <c r="O49" s="3" t="n">
-        <v>33.23</v>
+        <v>34.55</v>
       </c>
       <c r="P49" s="3" t="n">
-        <v>41.18</v>
+        <v>34.48</v>
       </c>
       <c r="Q49" s="3" t="n">
-        <v>48.43</v>
+        <v>40.6</v>
       </c>
       <c r="R49" s="3" t="n">
-        <v>56.38</v>
+        <v>48.49</v>
       </c>
       <c r="S49" s="3" t="n">
-        <v>56.34</v>
+        <v>51.16</v>
       </c>
       <c r="T49" s="3" t="n">
-        <v>54.1</v>
+        <v>49.56</v>
       </c>
       <c r="U49" s="3" t="n">
-        <v>49</v>
+        <v>50.62</v>
       </c>
       <c r="V49" s="3" t="n">
-        <v>37.73</v>
+        <v>50.18</v>
       </c>
       <c r="W49" s="3" t="n">
-        <v>35.06</v>
+        <v>47.16</v>
       </c>
       <c r="X49" s="3" t="n">
-        <v>32.18</v>
+        <v>37.32</v>
       </c>
       <c r="Y49" s="3" t="n">
-        <v>38.12</v>
+        <v>44.97</v>
       </c>
       <c r="Z49" s="3" t="n">
-        <v>40.77</v>
+        <v>41.19</v>
       </c>
     </row>
     <row r="50">
@@ -4601,73 +4601,73 @@
         <v>0.64</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.57</v>
+        <v>0.44</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0.55</v>
+        <v>0.4</v>
       </c>
       <c r="F51" s="3" t="n">
-        <v>1.12</v>
+        <v>0.54</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>1.96</v>
+        <v>1.18</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>2.19</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>1.32</v>
+        <v>0.45</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>0.8</v>
+        <v>0.14</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0.64</v>
+        <v>0.06</v>
       </c>
       <c r="L51" s="3" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="M51" s="3" t="n">
-        <v>0.92</v>
+        <v>0.59</v>
       </c>
       <c r="N51" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="O51" s="3" t="n">
-        <v>0.76</v>
+        <v>0.45</v>
       </c>
       <c r="P51" s="3" t="n">
-        <v>1.19</v>
+        <v>0.38</v>
       </c>
       <c r="Q51" s="3" t="n">
-        <v>1.31</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R51" s="3" t="n">
-        <v>1.41</v>
+        <v>0.44</v>
       </c>
       <c r="S51" s="3" t="n">
-        <v>1.69</v>
+        <v>0.97</v>
       </c>
       <c r="T51" s="3" t="n">
-        <v>1.57</v>
+        <v>1.09</v>
       </c>
       <c r="U51" s="3" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="V51" s="3" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="W51" s="3" t="n">
         <v>1.37</v>
       </c>
-      <c r="V51" s="3" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="W51" s="3" t="n">
-        <v>1.16</v>
-      </c>
       <c r="X51" s="3" t="n">
-        <v>0.8</v>
+        <v>1.27</v>
       </c>
       <c r="Y51" s="3" t="n">
-        <v>1.45</v>
+        <v>1.35</v>
       </c>
       <c r="Z51" s="3" t="n">
-        <v>1.26</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="52">
@@ -4784,7 +4784,7 @@
         <v>0</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J53" s="3" t="n">
         <v>0</v>
@@ -4856,70 +4856,70 @@
         <v>21.52</v>
       </c>
       <c r="E54" s="3" t="n">
-        <v>21.55</v>
+        <v>15.87</v>
       </c>
       <c r="F54" s="3" t="n">
-        <v>34.62</v>
+        <v>21.32</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>48.33</v>
+        <v>33.34</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>47.83</v>
+        <v>38.67</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>40.67</v>
+        <v>51.35</v>
       </c>
       <c r="J54" s="3" t="n">
-        <v>36.2</v>
+        <v>34.9</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>31.75</v>
+        <v>31.65</v>
       </c>
       <c r="L54" s="3" t="n">
-        <v>31.56</v>
+        <v>32.02</v>
       </c>
       <c r="M54" s="3" t="n">
-        <v>31.75</v>
+        <v>34.34</v>
       </c>
       <c r="N54" s="3" t="n">
-        <v>32.14</v>
+        <v>33.97</v>
       </c>
       <c r="O54" s="3" t="n">
-        <v>31.83</v>
+        <v>33.6</v>
       </c>
       <c r="P54" s="3" t="n">
-        <v>38.48</v>
+        <v>32.98</v>
       </c>
       <c r="Q54" s="3" t="n">
-        <v>45.4</v>
+        <v>38.71</v>
       </c>
       <c r="R54" s="3" t="n">
-        <v>52.65</v>
+        <v>46.25</v>
       </c>
       <c r="S54" s="3" t="n">
-        <v>51.22</v>
+        <v>47.17</v>
       </c>
       <c r="T54" s="3" t="n">
-        <v>49.41</v>
+        <v>45.68</v>
       </c>
       <c r="U54" s="3" t="n">
-        <v>44.97</v>
+        <v>46.12</v>
       </c>
       <c r="V54" s="3" t="n">
-        <v>34.11</v>
+        <v>45.73</v>
       </c>
       <c r="W54" s="3" t="n">
-        <v>32.44</v>
+        <v>44.16</v>
       </c>
       <c r="X54" s="3" t="n">
-        <v>31.5</v>
+        <v>36.16</v>
       </c>
       <c r="Y54" s="3" t="n">
-        <v>37.92</v>
+        <v>45.2</v>
       </c>
       <c r="Z54" s="3" t="n">
-        <v>40.81</v>
+        <v>41.19</v>
       </c>
     </row>
     <row r="55">
@@ -5024,70 +5024,70 @@
         <v>1.03</v>
       </c>
       <c r="E56" s="3" t="n">
-        <v>1.06</v>
+        <v>0.76</v>
       </c>
       <c r="F56" s="3" t="n">
-        <v>1.66</v>
+        <v>1.04</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>2.51</v>
+        <v>1.63</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>2.39</v>
+        <v>1.78</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>0.65</v>
+        <v>0</v>
       </c>
       <c r="J56" s="3" t="n">
-        <v>0.54</v>
+        <v>0</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>0.16</v>
+        <v>-0.19</v>
       </c>
       <c r="L56" s="3" t="n">
-        <v>-0.03</v>
+        <v>0.13</v>
       </c>
       <c r="M56" s="3" t="n">
-        <v>-0.06</v>
+        <v>0.1</v>
       </c>
       <c r="N56" s="3" t="n">
-        <v>-0.32</v>
+        <v>-0.17</v>
       </c>
       <c r="O56" s="3" t="n">
-        <v>-0.64</v>
+        <v>-0.5</v>
       </c>
       <c r="P56" s="3" t="n">
-        <v>-1.5</v>
+        <v>-1.12</v>
       </c>
       <c r="Q56" s="3" t="n">
-        <v>-1.73</v>
+        <v>-1.2</v>
       </c>
       <c r="R56" s="3" t="n">
-        <v>-2.32</v>
+        <v>-1.8</v>
       </c>
       <c r="S56" s="3" t="n">
-        <v>-3.43</v>
+        <v>-3.02</v>
       </c>
       <c r="T56" s="3" t="n">
-        <v>-3.11</v>
+        <v>-2.79</v>
       </c>
       <c r="U56" s="3" t="n">
-        <v>-2.65</v>
+        <v>-2.68</v>
       </c>
       <c r="V56" s="3" t="n">
-        <v>-2.18</v>
+        <v>-2.7</v>
       </c>
       <c r="W56" s="3" t="n">
-        <v>-1.46</v>
+        <v>-1.63</v>
       </c>
       <c r="X56" s="3" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="Y56" s="3" t="n">
-        <v>1.25</v>
+        <v>1.58</v>
       </c>
       <c r="Z56" s="3" t="n">
-        <v>1.31</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="57">
@@ -5204,7 +5204,7 @@
         <v>0</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J58" s="3" t="n">
         <v>0</v>
@@ -5273,73 +5273,73 @@
         <v>21.39</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>21.21</v>
+        <v>21.26</v>
       </c>
       <c r="E59" s="3" t="n">
-        <v>21.19</v>
+        <v>15.64</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>34.08</v>
+        <v>21.03</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>47.23</v>
+        <v>32.93</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>46.94</v>
+        <v>38.26</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>41.09</v>
+        <v>52.96</v>
       </c>
       <c r="J59" s="3" t="n">
-        <v>36.46</v>
+        <v>35.75</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>32.33</v>
+        <v>32.63</v>
       </c>
       <c r="L59" s="3" t="n">
-        <v>32.3</v>
+        <v>32.61</v>
       </c>
       <c r="M59" s="3" t="n">
-        <v>32.53</v>
+        <v>35.05</v>
       </c>
       <c r="N59" s="3" t="n">
-        <v>33.33</v>
+        <v>35.12</v>
       </c>
       <c r="O59" s="3" t="n">
-        <v>33.36</v>
+        <v>35.16</v>
       </c>
       <c r="P59" s="3" t="n">
+        <v>35.12</v>
+      </c>
+      <c r="Q59" s="3" t="n">
         <v>41.18</v>
       </c>
-      <c r="Q59" s="3" t="n">
-        <v>48.53</v>
-      </c>
       <c r="R59" s="3" t="n">
-        <v>56.96</v>
+        <v>49.74</v>
       </c>
       <c r="S59" s="3" t="n">
-        <v>56.63</v>
+        <v>51.95</v>
       </c>
       <c r="T59" s="3" t="n">
-        <v>54.38</v>
+        <v>50.18</v>
       </c>
       <c r="U59" s="3" t="n">
-        <v>49.25</v>
+        <v>50.52</v>
       </c>
       <c r="V59" s="3" t="n">
-        <v>37.61</v>
+        <v>50.13</v>
       </c>
       <c r="W59" s="3" t="n">
-        <v>35.17</v>
+        <v>47.4</v>
       </c>
       <c r="X59" s="3" t="n">
-        <v>32.18</v>
+        <v>36.97</v>
       </c>
       <c r="Y59" s="3" t="n">
-        <v>37.77</v>
+        <v>44.97</v>
       </c>
       <c r="Z59" s="3" t="n">
-        <v>40.6</v>
+        <v>40.64</v>
       </c>
     </row>
     <row r="60">
@@ -5441,70 +5441,70 @@
         <v>0.73</v>
       </c>
       <c r="D61" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="K61" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="L61" s="3" t="n">
         <v>0.72</v>
       </c>
-      <c r="E61" s="3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F61" s="3" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="G61" s="3" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="H61" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I61" s="3" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="J61" s="3" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K61" s="3" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="L61" s="3" t="n">
-        <v>0.71</v>
-      </c>
       <c r="M61" s="3" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="N61" s="3" t="n">
-        <v>0.87</v>
+        <v>0.98</v>
       </c>
       <c r="O61" s="3" t="n">
-        <v>0.9</v>
+        <v>1.05</v>
       </c>
       <c r="P61" s="3" t="n">
-        <v>1.19</v>
+        <v>1.02</v>
       </c>
       <c r="Q61" s="3" t="n">
-        <v>1.41</v>
+        <v>1.28</v>
       </c>
       <c r="R61" s="3" t="n">
-        <v>1.99</v>
+        <v>1.69</v>
       </c>
       <c r="S61" s="3" t="n">
-        <v>1.98</v>
+        <v>1.77</v>
       </c>
       <c r="T61" s="3" t="n">
-        <v>1.85</v>
+        <v>1.71</v>
       </c>
       <c r="U61" s="3" t="n">
-        <v>1.63</v>
+        <v>1.72</v>
       </c>
       <c r="V61" s="3" t="n">
-        <v>1.32</v>
+        <v>1.7</v>
       </c>
       <c r="W61" s="3" t="n">
-        <v>1.27</v>
+        <v>1.61</v>
       </c>
       <c r="X61" s="3" t="n">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="Y61" s="3" t="n">
-        <v>1.1</v>
+        <v>1.35</v>
       </c>
       <c r="Z61" s="3" t="n">
         <v>1.1</v>
@@ -5624,7 +5624,7 @@
         <v>0</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J63" s="3" t="n">
         <v>0</v>
@@ -5693,73 +5693,73 @@
         <v>21.66</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>21.48</v>
+        <v>21.5</v>
       </c>
       <c r="E64" s="3" t="n">
-        <v>21.44</v>
+        <v>15.8</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>34.51</v>
+        <v>21.27</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>47.87</v>
+        <v>33.31</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>47.63</v>
+        <v>38.75</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>41.69</v>
+        <v>53.54</v>
       </c>
       <c r="J64" s="3" t="n">
-        <v>36.95</v>
+        <v>36.2</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>32.77</v>
+        <v>33</v>
       </c>
       <c r="L64" s="3" t="n">
-        <v>32.77</v>
+        <v>33.02</v>
       </c>
       <c r="M64" s="3" t="n">
-        <v>33.03</v>
+        <v>35.45</v>
       </c>
       <c r="N64" s="3" t="n">
-        <v>33.89</v>
+        <v>35.6</v>
       </c>
       <c r="O64" s="3" t="n">
-        <v>33.92</v>
+        <v>35.6</v>
       </c>
       <c r="P64" s="3" t="n">
-        <v>41.74</v>
+        <v>35.6</v>
       </c>
       <c r="Q64" s="3" t="n">
-        <v>49.29</v>
+        <v>41.7</v>
       </c>
       <c r="R64" s="3" t="n">
-        <v>57.92</v>
+        <v>50.47</v>
       </c>
       <c r="S64" s="3" t="n">
-        <v>57.53</v>
+        <v>52.72</v>
       </c>
       <c r="T64" s="3" t="n">
-        <v>55.23</v>
+        <v>50.97</v>
       </c>
       <c r="U64" s="3" t="n">
-        <v>50.03</v>
+        <v>51.31</v>
       </c>
       <c r="V64" s="3" t="n">
-        <v>38.17</v>
+        <v>50.92</v>
       </c>
       <c r="W64" s="3" t="n">
-        <v>35.61</v>
+        <v>48.1</v>
       </c>
       <c r="X64" s="3" t="n">
-        <v>32.58</v>
+        <v>37.43</v>
       </c>
       <c r="Y64" s="3" t="n">
-        <v>38.2</v>
+        <v>45.58</v>
       </c>
       <c r="Z64" s="3" t="n">
-        <v>41.11</v>
+        <v>41.41</v>
       </c>
     </row>
     <row r="65">
@@ -5861,73 +5861,73 @@
         <v>1</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0.99</v>
+        <v>1.01</v>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>1.55</v>
+        <v>1</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>2.06</v>
+        <v>1.6</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>2.19</v>
+        <v>1.86</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>1.67</v>
+        <v>2.18</v>
       </c>
       <c r="J66" s="3" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>1.18</v>
+        <v>1.15</v>
       </c>
       <c r="L66" s="3" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="M66" s="3" t="n">
-        <v>1.22</v>
+        <v>1.21</v>
       </c>
       <c r="N66" s="3" t="n">
-        <v>1.42</v>
+        <v>1.46</v>
       </c>
       <c r="O66" s="3" t="n">
-        <v>1.46</v>
+        <v>1.5</v>
       </c>
       <c r="P66" s="3" t="n">
-        <v>1.75</v>
+        <v>1.5</v>
       </c>
       <c r="Q66" s="3" t="n">
-        <v>2.17</v>
+        <v>1.79</v>
       </c>
       <c r="R66" s="3" t="n">
-        <v>2.95</v>
+        <v>2.42</v>
       </c>
       <c r="S66" s="3" t="n">
-        <v>2.88</v>
+        <v>2.53</v>
       </c>
       <c r="T66" s="3" t="n">
-        <v>2.71</v>
+        <v>2.5</v>
       </c>
       <c r="U66" s="3" t="n">
-        <v>2.4</v>
+        <v>2.51</v>
       </c>
       <c r="V66" s="3" t="n">
-        <v>1.87</v>
+        <v>2.49</v>
       </c>
       <c r="W66" s="3" t="n">
-        <v>1.71</v>
+        <v>2.31</v>
       </c>
       <c r="X66" s="3" t="n">
-        <v>1.21</v>
+        <v>1.39</v>
       </c>
       <c r="Y66" s="3" t="n">
-        <v>1.53</v>
+        <v>1.96</v>
       </c>
       <c r="Z66" s="3" t="n">
-        <v>1.6</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="67">
@@ -6044,7 +6044,7 @@
         <v>0</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J68" s="3" t="n">
         <v>0</v>
@@ -6113,73 +6113,73 @@
         <v>55</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>21.8</v>
+        <v>21.82</v>
       </c>
       <c r="E69" s="3" t="n">
-        <v>21.75</v>
+        <v>16.05</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>34.95</v>
+        <v>21.59</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>48.43</v>
+        <v>33.8</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>48.13</v>
+        <v>75.2</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>42.04</v>
+        <v>54.18</v>
       </c>
       <c r="J69" s="3" t="n">
-        <v>37.26</v>
+        <v>36.5</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>33.04</v>
+        <v>33.31</v>
       </c>
       <c r="L69" s="3" t="n">
-        <v>33.01</v>
+        <v>33.33</v>
       </c>
       <c r="M69" s="3" t="n">
-        <v>33.24</v>
+        <v>35.82</v>
       </c>
       <c r="N69" s="3" t="n">
-        <v>34.17</v>
+        <v>35.97</v>
       </c>
       <c r="O69" s="3" t="n">
-        <v>34.21</v>
+        <v>36.01</v>
       </c>
       <c r="P69" s="3" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="Q69" s="3" t="n">
         <v>42.18</v>
       </c>
-      <c r="Q69" s="3" t="n">
-        <v>49.76</v>
-      </c>
       <c r="R69" s="3" t="n">
-        <v>58.47</v>
+        <v>51.06</v>
       </c>
       <c r="S69" s="3" t="n">
-        <v>58.08</v>
+        <v>53.27</v>
       </c>
       <c r="T69" s="3" t="n">
-        <v>55.82</v>
+        <v>51.51</v>
       </c>
       <c r="U69" s="3" t="n">
-        <v>50.56</v>
+        <v>51.86</v>
       </c>
       <c r="V69" s="3" t="n">
-        <v>38.53</v>
+        <v>51.4</v>
       </c>
       <c r="W69" s="3" t="n">
-        <v>36.06</v>
+        <v>48.66</v>
       </c>
       <c r="X69" s="3" t="n">
-        <v>32.85</v>
+        <v>37.75</v>
       </c>
       <c r="Y69" s="3" t="n">
-        <v>38.77</v>
+        <v>46.16</v>
       </c>
       <c r="Z69" s="3" t="n">
-        <v>41.45</v>
+        <v>41.54</v>
       </c>
     </row>
     <row r="70">
@@ -6281,73 +6281,73 @@
         <v>1.32</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>1.31</v>
+        <v>1.33</v>
       </c>
       <c r="E71" s="3" t="n">
-        <v>1.26</v>
+        <v>0.95</v>
       </c>
       <c r="F71" s="3" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="M71" s="3" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="N71" s="3" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="O71" s="3" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="P71" s="3" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="Q71" s="3" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R71" s="3" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="S71" s="3" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="T71" s="3" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="U71" s="3" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="V71" s="3" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="W71" s="3" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="X71" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Y71" s="3" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="Z71" s="3" t="n">
         <v>1.99</v>
-      </c>
-      <c r="G71" s="3" t="n">
-        <v>2.62</v>
-      </c>
-      <c r="H71" s="3" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="I71" s="3" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="J71" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K71" s="3" t="n">
-        <v>1.45</v>
-      </c>
-      <c r="L71" s="3" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="M71" s="3" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="N71" s="3" t="n">
-        <v>1.71</v>
-      </c>
-      <c r="O71" s="3" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="P71" s="3" t="n">
-        <v>2.19</v>
-      </c>
-      <c r="Q71" s="3" t="n">
-        <v>2.64</v>
-      </c>
-      <c r="R71" s="3" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="S71" s="3" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="T71" s="3" t="n">
-        <v>3.29</v>
-      </c>
-      <c r="U71" s="3" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="V71" s="3" t="n">
-        <v>2.23</v>
-      </c>
-      <c r="W71" s="3" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="X71" s="3" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="Y71" s="3" t="n">
-        <v>2.09</v>
-      </c>
-      <c r="Z71" s="3" t="n">
-        <v>1.95</v>
       </c>
     </row>
     <row r="72">
@@ -6377,7 +6377,7 @@
         <v>0</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>0</v>
+        <v>35.92</v>
       </c>
       <c r="I72" s="3" t="n">
         <v>0</v>
@@ -6464,7 +6464,7 @@
         <v>0</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J73" s="3" t="n">
         <v>0</v>
@@ -6533,70 +6533,70 @@
         <v>21.26</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>21.08</v>
+        <v>21.1</v>
       </c>
       <c r="E74" s="3" t="n">
-        <v>21.06</v>
+        <v>15.52</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>33.87</v>
+        <v>20.88</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>47.09</v>
+        <v>32.72</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>46.8</v>
+        <v>38.03</v>
       </c>
       <c r="I74" s="3" t="n">
+        <v>52.72</v>
+      </c>
+      <c r="J74" s="3" t="n">
+        <v>35.61</v>
+      </c>
+      <c r="K74" s="3" t="n">
+        <v>32.46</v>
+      </c>
+      <c r="L74" s="3" t="n">
+        <v>32.51</v>
+      </c>
+      <c r="M74" s="3" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="N74" s="3" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="O74" s="3" t="n">
+        <v>34.98</v>
+      </c>
+      <c r="P74" s="3" t="n">
+        <v>34.94</v>
+      </c>
+      <c r="Q74" s="3" t="n">
         <v>40.97</v>
       </c>
-      <c r="J74" s="3" t="n">
-        <v>36.35</v>
-      </c>
-      <c r="K74" s="3" t="n">
-        <v>32.23</v>
-      </c>
-      <c r="L74" s="3" t="n">
-        <v>32.2</v>
-      </c>
-      <c r="M74" s="3" t="n">
-        <v>32.43</v>
-      </c>
-      <c r="N74" s="3" t="n">
-        <v>33.23</v>
-      </c>
-      <c r="O74" s="3" t="n">
-        <v>33.23</v>
-      </c>
-      <c r="P74" s="3" t="n">
-        <v>41.01</v>
-      </c>
-      <c r="Q74" s="3" t="n">
-        <v>48.38</v>
-      </c>
       <c r="R74" s="3" t="n">
-        <v>56.78</v>
+        <v>49.49</v>
       </c>
       <c r="S74" s="3" t="n">
-        <v>56.46</v>
+        <v>51.74</v>
       </c>
       <c r="T74" s="3" t="n">
-        <v>54.21</v>
+        <v>50.02</v>
       </c>
       <c r="U74" s="3" t="n">
-        <v>49.1</v>
+        <v>50.36</v>
       </c>
       <c r="V74" s="3" t="n">
-        <v>37.53</v>
+        <v>49.97</v>
       </c>
       <c r="W74" s="3" t="n">
-        <v>35.06</v>
+        <v>47.21</v>
       </c>
       <c r="X74" s="3" t="n">
-        <v>32.08</v>
+        <v>36.82</v>
       </c>
       <c r="Y74" s="3" t="n">
-        <v>37.65</v>
+        <v>44.78</v>
       </c>
       <c r="Z74" s="3" t="n">
         <v>40.52</v>
@@ -6701,73 +6701,73 @@
         <v>0.6</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0.59</v>
+        <v>0.61</v>
       </c>
       <c r="E76" s="3" t="n">
-        <v>0.57</v>
+        <v>0.42</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>0.91</v>
+        <v>0.61</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>1.27</v>
+        <v>1.01</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>1.36</v>
+        <v>1.14</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.37</v>
       </c>
       <c r="J76" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.71</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>0.64</v>
+        <v>0.62</v>
       </c>
       <c r="L76" s="3" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="M76" s="3" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="N76" s="3" t="n">
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
       <c r="O76" s="3" t="n">
-        <v>0.76</v>
+        <v>0.87</v>
       </c>
       <c r="P76" s="3" t="n">
-        <v>1.03</v>
+        <v>0.84</v>
       </c>
       <c r="Q76" s="3" t="n">
-        <v>1.26</v>
+        <v>1.07</v>
       </c>
       <c r="R76" s="3" t="n">
-        <v>1.82</v>
+        <v>1.44</v>
       </c>
       <c r="S76" s="3" t="n">
-        <v>1.81</v>
+        <v>1.55</v>
       </c>
       <c r="T76" s="3" t="n">
-        <v>1.68</v>
+        <v>1.55</v>
       </c>
       <c r="U76" s="3" t="n">
-        <v>1.47</v>
+        <v>1.56</v>
       </c>
       <c r="V76" s="3" t="n">
-        <v>1.24</v>
+        <v>1.55</v>
       </c>
       <c r="W76" s="3" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="X76" s="3" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="Y76" s="3" t="n">
         <v>1.16</v>
       </c>
-      <c r="X76" s="3" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="Y76" s="3" t="n">
-        <v>0.98</v>
-      </c>
       <c r="Z76" s="3" t="n">
-        <v>1.01</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="77">
@@ -6884,7 +6884,7 @@
         <v>0</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J78" s="3" t="n">
         <v>0</v>
@@ -6956,70 +6956,70 @@
         <v>20.49</v>
       </c>
       <c r="E79" s="3" t="n">
-        <v>20.49</v>
+        <v>15.1</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>32.95</v>
+        <v>20.27</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>45.81</v>
+        <v>31.71</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>45.44</v>
+        <v>36.89</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>40.02</v>
+        <v>51.35</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>35.66</v>
+        <v>34.9</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>31.59</v>
+        <v>31.84</v>
       </c>
       <c r="L79" s="3" t="n">
-        <v>31.59</v>
+        <v>31.9</v>
       </c>
       <c r="M79" s="3" t="n">
-        <v>31.81</v>
+        <v>34.24</v>
       </c>
       <c r="N79" s="3" t="n">
-        <v>32.46</v>
+        <v>34.14</v>
       </c>
       <c r="O79" s="3" t="n">
-        <v>32.46</v>
+        <v>34.1</v>
       </c>
       <c r="P79" s="3" t="n">
-        <v>39.99</v>
+        <v>34.1</v>
       </c>
       <c r="Q79" s="3" t="n">
-        <v>47.13</v>
+        <v>39.91</v>
       </c>
       <c r="R79" s="3" t="n">
-        <v>54.97</v>
+        <v>48.05</v>
       </c>
       <c r="S79" s="3" t="n">
-        <v>54.65</v>
+        <v>50.18</v>
       </c>
       <c r="T79" s="3" t="n">
-        <v>52.53</v>
+        <v>48.47</v>
       </c>
       <c r="U79" s="3" t="n">
-        <v>47.63</v>
+        <v>48.8</v>
       </c>
       <c r="V79" s="3" t="n">
-        <v>36.3</v>
+        <v>48.42</v>
       </c>
       <c r="W79" s="3" t="n">
-        <v>33.9</v>
+        <v>45.79</v>
       </c>
       <c r="X79" s="3" t="n">
-        <v>31.37</v>
+        <v>36.05</v>
       </c>
       <c r="Y79" s="3" t="n">
-        <v>36.67</v>
+        <v>43.62</v>
       </c>
       <c r="Z79" s="3" t="n">
-        <v>39.5</v>
+        <v>39.54</v>
       </c>
     </row>
     <row r="80">
@@ -7304,7 +7304,7 @@
         <v>0</v>
       </c>
       <c r="I83" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J83" s="3" t="n">
         <v>0</v>
@@ -7373,73 +7373,73 @@
         <v>21.37</v>
       </c>
       <c r="D84" s="3" t="n">
-        <v>21.19</v>
+        <v>21.23</v>
       </c>
       <c r="E84" s="3" t="n">
-        <v>21.24</v>
+        <v>15.65</v>
       </c>
       <c r="F84" s="3" t="n">
-        <v>33.97</v>
+        <v>21.03</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>47.77</v>
+        <v>33</v>
       </c>
       <c r="H84" s="3" t="n">
-        <v>47.73</v>
+        <v>38.54</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>40.84</v>
+        <v>50.44</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>36.35</v>
+        <v>34.01</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>32.01</v>
+        <v>31.13</v>
       </c>
       <c r="L84" s="3" t="n">
-        <v>31.75</v>
+        <v>32.35</v>
       </c>
       <c r="M84" s="3" t="n">
-        <v>31.81</v>
+        <v>34.62</v>
       </c>
       <c r="N84" s="3" t="n">
-        <v>32.08</v>
+        <v>34.14</v>
       </c>
       <c r="O84" s="3" t="n">
-        <v>31.83</v>
+        <v>33.9</v>
       </c>
       <c r="P84" s="3" t="n">
-        <v>38.78</v>
+        <v>33.63</v>
       </c>
       <c r="Q84" s="3" t="n">
-        <v>45.71</v>
+        <v>39.47</v>
       </c>
       <c r="R84" s="3" t="n">
-        <v>53.06</v>
+        <v>47.34</v>
       </c>
       <c r="S84" s="3" t="n">
-        <v>50.55</v>
+        <v>47.08</v>
       </c>
       <c r="T84" s="3" t="n">
-        <v>49.23</v>
+        <v>45.81</v>
       </c>
       <c r="U84" s="3" t="n">
-        <v>44.97</v>
+        <v>46.52</v>
       </c>
       <c r="V84" s="3" t="n">
-        <v>34.05</v>
+        <v>46.25</v>
       </c>
       <c r="W84" s="3" t="n">
-        <v>31.95</v>
+        <v>44.24</v>
       </c>
       <c r="X84" s="3" t="n">
-        <v>31.4</v>
+        <v>36.82</v>
       </c>
       <c r="Y84" s="3" t="n">
-        <v>37.65</v>
+        <v>45.53</v>
       </c>
       <c r="Z84" s="3" t="n">
-        <v>40.48</v>
+        <v>41.32</v>
       </c>
     </row>
     <row r="85">
@@ -7541,73 +7541,73 @@
         <v>0.71</v>
       </c>
       <c r="D86" s="3" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="E86" s="3" t="n">
-        <v>0.74</v>
+        <v>0.55</v>
       </c>
       <c r="F86" s="3" t="n">
-        <v>1.02</v>
+        <v>0.76</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>1.96</v>
+        <v>1.29</v>
       </c>
       <c r="H86" s="3" t="n">
-        <v>2.29</v>
+        <v>1.66</v>
       </c>
       <c r="I86" s="3" t="n">
-        <v>0.82</v>
+        <v>-0.91</v>
       </c>
       <c r="J86" s="3" t="n">
-        <v>0.6899999999999999</v>
+        <v>-0.88</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>0.42</v>
+        <v>-0.72</v>
       </c>
       <c r="L86" s="3" t="n">
-        <v>0.16</v>
+        <v>0.45</v>
       </c>
       <c r="M86" s="3" t="n">
-        <v>0</v>
+        <v>0.38</v>
       </c>
       <c r="N86" s="3" t="n">
-        <v>-0.38</v>
+        <v>0</v>
       </c>
       <c r="O86" s="3" t="n">
-        <v>-0.64</v>
+        <v>-0.2</v>
       </c>
       <c r="P86" s="3" t="n">
-        <v>-1.2</v>
+        <v>-0.47</v>
       </c>
       <c r="Q86" s="3" t="n">
-        <v>-1.42</v>
+        <v>-0.43</v>
       </c>
       <c r="R86" s="3" t="n">
-        <v>-1.91</v>
+        <v>-0.71</v>
       </c>
       <c r="S86" s="3" t="n">
-        <v>-4.09</v>
+        <v>-3.11</v>
       </c>
       <c r="T86" s="3" t="n">
-        <v>-3.3</v>
+        <v>-2.66</v>
       </c>
       <c r="U86" s="3" t="n">
-        <v>-2.65</v>
+        <v>-2.28</v>
       </c>
       <c r="V86" s="3" t="n">
-        <v>-2.25</v>
+        <v>-2.17</v>
       </c>
       <c r="W86" s="3" t="n">
-        <v>-1.95</v>
+        <v>-1.55</v>
       </c>
       <c r="X86" s="3" t="n">
-        <v>0.03</v>
+        <v>0.77</v>
       </c>
       <c r="Y86" s="3" t="n">
-        <v>0.98</v>
+        <v>1.91</v>
       </c>
       <c r="Z86" s="3" t="n">
-        <v>0.97</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="87">
@@ -7724,7 +7724,7 @@
         <v>0</v>
       </c>
       <c r="I88" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J88" s="3" t="n">
         <v>0</v>
@@ -7796,70 +7796,70 @@
         <v>60.2</v>
       </c>
       <c r="E89" s="3" t="n">
-        <v>20.68</v>
+        <v>57</v>
       </c>
       <c r="F89" s="3" t="n">
-        <v>33.02</v>
+        <v>59</v>
       </c>
       <c r="G89" s="3" t="n">
-        <v>45.23</v>
+        <v>66</v>
       </c>
       <c r="H89" s="3" t="n">
-        <v>44.59</v>
+        <v>98.2</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>39.51</v>
+        <v>87.61</v>
       </c>
       <c r="J89" s="3" t="n">
-        <v>35.2</v>
+        <v>34.55</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>31.31</v>
+        <v>31.5</v>
       </c>
       <c r="L89" s="3" t="n">
-        <v>31.31</v>
+        <v>31.58</v>
       </c>
       <c r="M89" s="3" t="n">
-        <v>31.59</v>
+        <v>34</v>
       </c>
       <c r="N89" s="3" t="n">
-        <v>32.27</v>
+        <v>33.97</v>
       </c>
       <c r="O89" s="3" t="n">
-        <v>32.27</v>
+        <v>33.97</v>
       </c>
       <c r="P89" s="3" t="n">
-        <v>39.55</v>
+        <v>33.83</v>
       </c>
       <c r="Q89" s="3" t="n">
-        <v>46.29</v>
+        <v>39.59</v>
       </c>
       <c r="R89" s="3" t="n">
-        <v>53.73</v>
+        <v>47.29</v>
       </c>
       <c r="S89" s="3" t="n">
-        <v>53.53</v>
+        <v>49.2</v>
       </c>
       <c r="T89" s="3" t="n">
-        <v>51.15</v>
+        <v>47.24</v>
       </c>
       <c r="U89" s="3" t="n">
-        <v>46.29</v>
+        <v>47.38</v>
       </c>
       <c r="V89" s="3" t="n">
-        <v>35.65</v>
+        <v>46.97</v>
       </c>
       <c r="W89" s="3" t="n">
-        <v>33.7</v>
+        <v>44.76</v>
       </c>
       <c r="X89" s="3" t="n">
-        <v>31.22</v>
+        <v>35.55</v>
       </c>
       <c r="Y89" s="3" t="n">
-        <v>36.2</v>
+        <v>42.93</v>
       </c>
       <c r="Z89" s="3" t="n">
-        <v>39.15</v>
+        <v>38.92</v>
       </c>
     </row>
     <row r="90">
@@ -7961,73 +7961,73 @@
         <v>0.02</v>
       </c>
       <c r="D91" s="3" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="E91" s="3" t="n">
-        <v>0.19</v>
+        <v>0.09</v>
       </c>
       <c r="F91" s="3" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.18</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>-0.59</v>
+        <v>-0.13</v>
       </c>
       <c r="H91" s="3" t="n">
-        <v>-0.85</v>
+        <v>-0.26</v>
       </c>
       <c r="I91" s="3" t="n">
-        <v>-0.51</v>
+        <v>-0.39</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>-0.46</v>
+        <v>-0.35</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.35</v>
       </c>
       <c r="L91" s="3" t="n">
-        <v>-0.28</v>
+        <v>-0.32</v>
       </c>
       <c r="M91" s="3" t="n">
-        <v>-0.22</v>
+        <v>-0.24</v>
       </c>
       <c r="N91" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.17</v>
       </c>
       <c r="O91" s="3" t="n">
-        <v>-0.19</v>
+        <v>-0.14</v>
       </c>
       <c r="P91" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.27</v>
       </c>
       <c r="Q91" s="3" t="n">
-        <v>-0.83</v>
+        <v>-0.32</v>
       </c>
       <c r="R91" s="3" t="n">
-        <v>-1.24</v>
+        <v>-0.76</v>
       </c>
       <c r="S91" s="3" t="n">
-        <v>-1.12</v>
+        <v>-0.98</v>
       </c>
       <c r="T91" s="3" t="n">
-        <v>-1.38</v>
+        <v>-1.23</v>
       </c>
       <c r="U91" s="3" t="n">
-        <v>-1.34</v>
+        <v>-1.42</v>
       </c>
       <c r="V91" s="3" t="n">
-        <v>-0.64</v>
+        <v>-1.46</v>
       </c>
       <c r="W91" s="3" t="n">
-        <v>-0.2</v>
+        <v>-1.03</v>
       </c>
       <c r="X91" s="3" t="n">
-        <v>-0.16</v>
+        <v>-0.5</v>
       </c>
       <c r="Y91" s="3" t="n">
-        <v>-0.47</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="Z91" s="3" t="n">
-        <v>-0.35</v>
+        <v>-0.62</v>
       </c>
     </row>
     <row r="92">
@@ -8045,22 +8045,22 @@
         <v>42.51</v>
       </c>
       <c r="D92" s="3" t="n">
-        <v>39.54</v>
+        <v>39.58</v>
       </c>
       <c r="E92" s="3" t="n">
-        <v>0</v>
+        <v>41.8</v>
       </c>
       <c r="F92" s="3" t="n">
-        <v>0</v>
+        <v>38.54</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>0</v>
+        <v>34.42</v>
       </c>
       <c r="H92" s="3" t="n">
-        <v>0</v>
+        <v>61.57</v>
       </c>
       <c r="I92" s="3" t="n">
-        <v>0</v>
+        <v>36.65</v>
       </c>
       <c r="J92" s="3" t="n">
         <v>0</v>
@@ -8144,7 +8144,7 @@
         <v>0</v>
       </c>
       <c r="I93" s="3" t="n">
-        <v>0</v>
+        <v>7.08</v>
       </c>
       <c r="J93" s="3" t="n">
         <v>0</v>

</xml_diff>